<commit_message>
Give the fixture continuous variables
The two datasets nearest the fixture size carried no numeric measurement at
all -- zero numeric values in any of 192 columns -- which left the cutoff and
correlation tabs with nothing to act on. They could not be tested, or even
demonstrated, against data-sample. Age, BMI, adipocyte size and adipocyte
score now get synthetic values in plausible ranges, in columns that already
exist.

check_fixtures.R requires at least two fully numeric columns, and was proved
able to fail by removing them: a fixture without them lets those tabs pass
every test by never having anything to do.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-sample/Metadata.xlsx
+++ b/data-sample/Metadata.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6144" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6020" uniqueCount="243">
   <si>
     <t>TsengID</t>
   </si>
@@ -1721,14 +1721,14 @@
       <c r="R2" t="s">
         <v>198</v>
       </c>
-      <c r="S2" t="s">
-        <v>198</v>
+      <c r="S2">
+        <v>58.18</v>
       </c>
       <c r="T2" t="s">
         <v>198</v>
       </c>
-      <c r="U2" t="s">
-        <v>198</v>
+      <c r="U2">
+        <v>53.82</v>
       </c>
       <c r="V2" t="s">
         <v>198</v>
@@ -1736,8 +1736,8 @@
       <c r="W2" t="s">
         <v>198</v>
       </c>
-      <c r="X2" t="s">
-        <v>198</v>
+      <c r="X2">
+        <v>0.13</v>
       </c>
       <c r="Y2" t="s">
         <v>198</v>
@@ -1934,8 +1934,8 @@
       <c r="CK2" t="s">
         <v>198</v>
       </c>
-      <c r="CL2" t="s">
-        <v>198</v>
+      <c r="CL2">
+        <v>39.75</v>
       </c>
       <c r="CM2" t="s">
         <v>198</v>
@@ -2299,14 +2299,14 @@
       <c r="R3" t="s">
         <v>198</v>
       </c>
-      <c r="S3" t="s">
-        <v>198</v>
+      <c r="S3">
+        <v>115.79</v>
       </c>
       <c r="T3" t="s">
         <v>198</v>
       </c>
-      <c r="U3" t="s">
-        <v>198</v>
+      <c r="U3">
+        <v>66.40000000000001</v>
       </c>
       <c r="V3" t="s">
         <v>198</v>
@@ -2314,8 +2314,8 @@
       <c r="W3" t="s">
         <v>198</v>
       </c>
-      <c r="X3" t="s">
-        <v>198</v>
+      <c r="X3">
+        <v>0.32</v>
       </c>
       <c r="Y3" t="s">
         <v>198</v>
@@ -2512,8 +2512,8 @@
       <c r="CK3" t="s">
         <v>198</v>
       </c>
-      <c r="CL3" t="s">
-        <v>198</v>
+      <c r="CL3">
+        <v>24.96</v>
       </c>
       <c r="CM3" t="s">
         <v>198</v>
@@ -2877,14 +2877,14 @@
       <c r="R4" t="s">
         <v>198</v>
       </c>
-      <c r="S4" t="s">
-        <v>198</v>
+      <c r="S4">
+        <v>131.49</v>
       </c>
       <c r="T4" t="s">
         <v>198</v>
       </c>
-      <c r="U4" t="s">
-        <v>198</v>
+      <c r="U4">
+        <v>24.95</v>
       </c>
       <c r="V4" t="s">
         <v>198</v>
@@ -2892,8 +2892,8 @@
       <c r="W4" t="s">
         <v>198</v>
       </c>
-      <c r="X4" t="s">
-        <v>198</v>
+      <c r="X4">
+        <v>0.1</v>
       </c>
       <c r="Y4" t="s">
         <v>198</v>
@@ -3090,8 +3090,8 @@
       <c r="CK4" t="s">
         <v>198</v>
       </c>
-      <c r="CL4" t="s">
-        <v>198</v>
+      <c r="CL4">
+        <v>21.74</v>
       </c>
       <c r="CM4" t="s">
         <v>198</v>
@@ -3455,14 +3455,14 @@
       <c r="R5" t="s">
         <v>198</v>
       </c>
-      <c r="S5" t="s">
-        <v>198</v>
+      <c r="S5">
+        <v>64.09999999999999</v>
       </c>
       <c r="T5" t="s">
         <v>198</v>
       </c>
-      <c r="U5" t="s">
-        <v>198</v>
+      <c r="U5">
+        <v>25.19</v>
       </c>
       <c r="V5" t="s">
         <v>198</v>
@@ -3470,8 +3470,8 @@
       <c r="W5" t="s">
         <v>198</v>
       </c>
-      <c r="X5" t="s">
-        <v>198</v>
+      <c r="X5">
+        <v>0.47</v>
       </c>
       <c r="Y5" t="s">
         <v>198</v>
@@ -3668,8 +3668,8 @@
       <c r="CK5" t="s">
         <v>198</v>
       </c>
-      <c r="CL5" t="s">
-        <v>198</v>
+      <c r="CL5">
+        <v>34.73</v>
       </c>
       <c r="CM5" t="s">
         <v>198</v>
@@ -4033,14 +4033,14 @@
       <c r="R6" t="s">
         <v>198</v>
       </c>
-      <c r="S6" t="s">
-        <v>198</v>
+      <c r="S6">
+        <v>66.72</v>
       </c>
       <c r="T6" t="s">
         <v>198</v>
       </c>
-      <c r="U6" t="s">
-        <v>198</v>
+      <c r="U6">
+        <v>20.77</v>
       </c>
       <c r="V6" t="s">
         <v>198</v>
@@ -4048,8 +4048,8 @@
       <c r="W6" t="s">
         <v>198</v>
       </c>
-      <c r="X6" t="s">
-        <v>198</v>
+      <c r="X6">
+        <v>0.4</v>
       </c>
       <c r="Y6" t="s">
         <v>198</v>
@@ -4246,8 +4246,8 @@
       <c r="CK6" t="s">
         <v>198</v>
       </c>
-      <c r="CL6" t="s">
-        <v>198</v>
+      <c r="CL6">
+        <v>27.94</v>
       </c>
       <c r="CM6" t="s">
         <v>198</v>
@@ -4611,14 +4611,14 @@
       <c r="R7" t="s">
         <v>198</v>
       </c>
-      <c r="S7" t="s">
-        <v>198</v>
+      <c r="S7">
+        <v>73.58</v>
       </c>
       <c r="T7" t="s">
         <v>198</v>
       </c>
-      <c r="U7" t="s">
-        <v>198</v>
+      <c r="U7">
+        <v>31.06</v>
       </c>
       <c r="V7" t="s">
         <v>198</v>
@@ -4626,8 +4626,8 @@
       <c r="W7" t="s">
         <v>198</v>
       </c>
-      <c r="X7" t="s">
-        <v>198</v>
+      <c r="X7">
+        <v>0.47</v>
       </c>
       <c r="Y7" t="s">
         <v>198</v>
@@ -4824,8 +4824,8 @@
       <c r="CK7" t="s">
         <v>198</v>
       </c>
-      <c r="CL7" t="s">
-        <v>198</v>
+      <c r="CL7">
+        <v>19.01</v>
       </c>
       <c r="CM7" t="s">
         <v>198</v>
@@ -5189,14 +5189,14 @@
       <c r="R8" t="s">
         <v>198</v>
       </c>
-      <c r="S8" t="s">
-        <v>198</v>
+      <c r="S8">
+        <v>91.76000000000001</v>
       </c>
       <c r="T8" t="s">
         <v>198</v>
       </c>
-      <c r="U8" t="s">
-        <v>198</v>
+      <c r="U8">
+        <v>37.1</v>
       </c>
       <c r="V8" t="s">
         <v>198</v>
@@ -5204,8 +5204,8 @@
       <c r="W8" t="s">
         <v>198</v>
       </c>
-      <c r="X8" t="s">
-        <v>198</v>
+      <c r="X8">
+        <v>0.88</v>
       </c>
       <c r="Y8" t="s">
         <v>198</v>
@@ -5402,8 +5402,8 @@
       <c r="CK8" t="s">
         <v>198</v>
       </c>
-      <c r="CL8" t="s">
-        <v>198</v>
+      <c r="CL8">
+        <v>39.6</v>
       </c>
       <c r="CM8" t="s">
         <v>198</v>
@@ -5767,14 +5767,14 @@
       <c r="R9" t="s">
         <v>198</v>
       </c>
-      <c r="S9" t="s">
-        <v>198</v>
+      <c r="S9">
+        <v>94.93000000000001</v>
       </c>
       <c r="T9" t="s">
         <v>198</v>
       </c>
-      <c r="U9" t="s">
-        <v>198</v>
+      <c r="U9">
+        <v>64.44</v>
       </c>
       <c r="V9" t="s">
         <v>198</v>
@@ -5782,8 +5782,8 @@
       <c r="W9" t="s">
         <v>198</v>
       </c>
-      <c r="X9" t="s">
-        <v>198</v>
+      <c r="X9">
+        <v>0.1</v>
       </c>
       <c r="Y9" t="s">
         <v>198</v>
@@ -5980,8 +5980,8 @@
       <c r="CK9" t="s">
         <v>198</v>
       </c>
-      <c r="CL9" t="s">
-        <v>198</v>
+      <c r="CL9">
+        <v>21.76</v>
       </c>
       <c r="CM9" t="s">
         <v>198</v>
@@ -6345,14 +6345,14 @@
       <c r="R10" t="s">
         <v>198</v>
       </c>
-      <c r="S10" t="s">
-        <v>198</v>
+      <c r="S10">
+        <v>65.28</v>
       </c>
       <c r="T10" t="s">
         <v>198</v>
       </c>
-      <c r="U10" t="s">
-        <v>198</v>
+      <c r="U10">
+        <v>26.62</v>
       </c>
       <c r="V10" t="s">
         <v>198</v>
@@ -6360,8 +6360,8 @@
       <c r="W10" t="s">
         <v>198</v>
       </c>
-      <c r="X10" t="s">
-        <v>198</v>
+      <c r="X10">
+        <v>0.28</v>
       </c>
       <c r="Y10" t="s">
         <v>198</v>
@@ -6558,8 +6558,8 @@
       <c r="CK10" t="s">
         <v>198</v>
       </c>
-      <c r="CL10" t="s">
-        <v>198</v>
+      <c r="CL10">
+        <v>36.7</v>
       </c>
       <c r="CM10" t="s">
         <v>198</v>
@@ -6923,14 +6923,14 @@
       <c r="R11" t="s">
         <v>198</v>
       </c>
-      <c r="S11" t="s">
-        <v>198</v>
+      <c r="S11">
+        <v>74.52</v>
       </c>
       <c r="T11" t="s">
         <v>198</v>
       </c>
-      <c r="U11" t="s">
-        <v>198</v>
+      <c r="U11">
+        <v>59.52</v>
       </c>
       <c r="V11" t="s">
         <v>198</v>
@@ -6938,8 +6938,8 @@
       <c r="W11" t="s">
         <v>198</v>
       </c>
-      <c r="X11" t="s">
-        <v>198</v>
+      <c r="X11">
+        <v>0.43</v>
       </c>
       <c r="Y11" t="s">
         <v>198</v>
@@ -7136,8 +7136,8 @@
       <c r="CK11" t="s">
         <v>198</v>
       </c>
-      <c r="CL11" t="s">
-        <v>198</v>
+      <c r="CL11">
+        <v>27.16</v>
       </c>
       <c r="CM11" t="s">
         <v>198</v>
@@ -7501,14 +7501,14 @@
       <c r="R12" t="s">
         <v>198</v>
       </c>
-      <c r="S12" t="s">
-        <v>198</v>
+      <c r="S12">
+        <v>77.11</v>
       </c>
       <c r="T12" t="s">
         <v>198</v>
       </c>
-      <c r="U12" t="s">
-        <v>198</v>
+      <c r="U12">
+        <v>59.32</v>
       </c>
       <c r="V12" t="s">
         <v>198</v>
@@ -7516,8 +7516,8 @@
       <c r="W12" t="s">
         <v>198</v>
       </c>
-      <c r="X12" t="s">
-        <v>198</v>
+      <c r="X12">
+        <v>0.05</v>
       </c>
       <c r="Y12" t="s">
         <v>198</v>
@@ -7714,8 +7714,8 @@
       <c r="CK12" t="s">
         <v>198</v>
       </c>
-      <c r="CL12" t="s">
-        <v>198</v>
+      <c r="CL12">
+        <v>37.74</v>
       </c>
       <c r="CM12" t="s">
         <v>198</v>
@@ -8079,14 +8079,14 @@
       <c r="R13" t="s">
         <v>198</v>
       </c>
-      <c r="S13" t="s">
-        <v>198</v>
+      <c r="S13">
+        <v>37.15</v>
       </c>
       <c r="T13" t="s">
         <v>198</v>
       </c>
-      <c r="U13" t="s">
-        <v>198</v>
+      <c r="U13">
+        <v>29.31</v>
       </c>
       <c r="V13" t="s">
         <v>198</v>
@@ -8094,8 +8094,8 @@
       <c r="W13" t="s">
         <v>198</v>
       </c>
-      <c r="X13" t="s">
-        <v>198</v>
+      <c r="X13">
+        <v>0.5600000000000001</v>
       </c>
       <c r="Y13" t="s">
         <v>198</v>
@@ -8292,8 +8292,8 @@
       <c r="CK13" t="s">
         <v>198</v>
       </c>
-      <c r="CL13" t="s">
-        <v>198</v>
+      <c r="CL13">
+        <v>33.28</v>
       </c>
       <c r="CM13" t="s">
         <v>198</v>
@@ -8657,14 +8657,14 @@
       <c r="R14" t="s">
         <v>198</v>
       </c>
-      <c r="S14" t="s">
-        <v>198</v>
+      <c r="S14">
+        <v>31.52</v>
       </c>
       <c r="T14" t="s">
         <v>198</v>
       </c>
-      <c r="U14" t="s">
-        <v>198</v>
+      <c r="U14">
+        <v>23.34</v>
       </c>
       <c r="V14" t="s">
         <v>198</v>
@@ -8672,8 +8672,8 @@
       <c r="W14" t="s">
         <v>198</v>
       </c>
-      <c r="X14" t="s">
-        <v>198</v>
+      <c r="X14">
+        <v>0.12</v>
       </c>
       <c r="Y14" t="s">
         <v>198</v>
@@ -8870,8 +8870,8 @@
       <c r="CK14" t="s">
         <v>198</v>
       </c>
-      <c r="CL14" t="s">
-        <v>198</v>
+      <c r="CL14">
+        <v>33.3</v>
       </c>
       <c r="CM14" t="s">
         <v>198</v>
@@ -9235,14 +9235,14 @@
       <c r="R15" t="s">
         <v>198</v>
       </c>
-      <c r="S15" t="s">
-        <v>198</v>
+      <c r="S15">
+        <v>87.98</v>
       </c>
       <c r="T15" t="s">
         <v>198</v>
       </c>
-      <c r="U15" t="s">
-        <v>198</v>
+      <c r="U15">
+        <v>39.76</v>
       </c>
       <c r="V15" t="s">
         <v>198</v>
@@ -9250,8 +9250,8 @@
       <c r="W15" t="s">
         <v>198</v>
       </c>
-      <c r="X15" t="s">
-        <v>198</v>
+      <c r="X15">
+        <v>0.25</v>
       </c>
       <c r="Y15" t="s">
         <v>198</v>
@@ -9448,8 +9448,8 @@
       <c r="CK15" t="s">
         <v>198</v>
       </c>
-      <c r="CL15" t="s">
-        <v>198</v>
+      <c r="CL15">
+        <v>31.17</v>
       </c>
       <c r="CM15" t="s">
         <v>198</v>
@@ -9813,14 +9813,14 @@
       <c r="R16" t="s">
         <v>198</v>
       </c>
-      <c r="S16" t="s">
-        <v>198</v>
+      <c r="S16">
+        <v>109.38</v>
       </c>
       <c r="T16" t="s">
         <v>198</v>
       </c>
-      <c r="U16" t="s">
-        <v>198</v>
+      <c r="U16">
+        <v>46.54</v>
       </c>
       <c r="V16" t="s">
         <v>198</v>
@@ -9828,8 +9828,8 @@
       <c r="W16" t="s">
         <v>198</v>
       </c>
-      <c r="X16" t="s">
-        <v>198</v>
+      <c r="X16">
+        <v>0.77</v>
       </c>
       <c r="Y16" t="s">
         <v>198</v>
@@ -10026,8 +10026,8 @@
       <c r="CK16" t="s">
         <v>198</v>
       </c>
-      <c r="CL16" t="s">
-        <v>198</v>
+      <c r="CL16">
+        <v>27.37</v>
       </c>
       <c r="CM16" t="s">
         <v>198</v>
@@ -10391,14 +10391,14 @@
       <c r="R17" t="s">
         <v>198</v>
       </c>
-      <c r="S17" t="s">
-        <v>198</v>
+      <c r="S17">
+        <v>104.31</v>
       </c>
       <c r="T17" t="s">
         <v>198</v>
       </c>
-      <c r="U17" t="s">
-        <v>198</v>
+      <c r="U17">
+        <v>57.92</v>
       </c>
       <c r="V17" t="s">
         <v>198</v>
@@ -10406,8 +10406,8 @@
       <c r="W17" t="s">
         <v>198</v>
       </c>
-      <c r="X17" t="s">
-        <v>198</v>
+      <c r="X17">
+        <v>0.52</v>
       </c>
       <c r="Y17" t="s">
         <v>198</v>
@@ -10604,8 +10604,8 @@
       <c r="CK17" t="s">
         <v>198</v>
       </c>
-      <c r="CL17" t="s">
-        <v>198</v>
+      <c r="CL17">
+        <v>32.81</v>
       </c>
       <c r="CM17" t="s">
         <v>198</v>
@@ -10969,14 +10969,14 @@
       <c r="R18" t="s">
         <v>198</v>
       </c>
-      <c r="S18" t="s">
-        <v>198</v>
+      <c r="S18">
+        <v>136.72</v>
       </c>
       <c r="T18" t="s">
         <v>198</v>
       </c>
-      <c r="U18" t="s">
-        <v>198</v>
+      <c r="U18">
+        <v>25.71</v>
       </c>
       <c r="V18" t="s">
         <v>198</v>
@@ -10984,8 +10984,8 @@
       <c r="W18" t="s">
         <v>198</v>
       </c>
-      <c r="X18" t="s">
-        <v>198</v>
+      <c r="X18">
+        <v>0.1</v>
       </c>
       <c r="Y18" t="s">
         <v>198</v>
@@ -11182,8 +11182,8 @@
       <c r="CK18" t="s">
         <v>198</v>
       </c>
-      <c r="CL18" t="s">
-        <v>198</v>
+      <c r="CL18">
+        <v>19.65</v>
       </c>
       <c r="CM18" t="s">
         <v>198</v>
@@ -11547,14 +11547,14 @@
       <c r="R19" t="s">
         <v>198</v>
       </c>
-      <c r="S19" t="s">
-        <v>198</v>
+      <c r="S19">
+        <v>142.87</v>
       </c>
       <c r="T19" t="s">
         <v>198</v>
       </c>
-      <c r="U19" t="s">
-        <v>198</v>
+      <c r="U19">
+        <v>56.2</v>
       </c>
       <c r="V19" t="s">
         <v>198</v>
@@ -11562,8 +11562,8 @@
       <c r="W19" t="s">
         <v>198</v>
       </c>
-      <c r="X19" t="s">
-        <v>198</v>
+      <c r="X19">
+        <v>0.76</v>
       </c>
       <c r="Y19" t="s">
         <v>198</v>
@@ -11760,8 +11760,8 @@
       <c r="CK19" t="s">
         <v>198</v>
       </c>
-      <c r="CL19" t="s">
-        <v>198</v>
+      <c r="CL19">
+        <v>39.53</v>
       </c>
       <c r="CM19" t="s">
         <v>198</v>
@@ -12125,14 +12125,14 @@
       <c r="R20" t="s">
         <v>198</v>
       </c>
-      <c r="S20" t="s">
-        <v>198</v>
+      <c r="S20">
+        <v>119.52</v>
       </c>
       <c r="T20" t="s">
         <v>198</v>
       </c>
-      <c r="U20" t="s">
-        <v>198</v>
+      <c r="U20">
+        <v>69.36</v>
       </c>
       <c r="V20" t="s">
         <v>198</v>
@@ -12140,8 +12140,8 @@
       <c r="W20" t="s">
         <v>198</v>
       </c>
-      <c r="X20" t="s">
-        <v>198</v>
+      <c r="X20">
+        <v>0.4</v>
       </c>
       <c r="Y20" t="s">
         <v>198</v>
@@ -12338,8 +12338,8 @@
       <c r="CK20" t="s">
         <v>198</v>
       </c>
-      <c r="CL20" t="s">
-        <v>198</v>
+      <c r="CL20">
+        <v>29.14</v>
       </c>
       <c r="CM20" t="s">
         <v>198</v>
@@ -12703,14 +12703,14 @@
       <c r="R21" t="s">
         <v>198</v>
       </c>
-      <c r="S21" t="s">
-        <v>198</v>
+      <c r="S21">
+        <v>101.52</v>
       </c>
       <c r="T21" t="s">
         <v>198</v>
       </c>
-      <c r="U21" t="s">
-        <v>198</v>
+      <c r="U21">
+        <v>55.38</v>
       </c>
       <c r="V21" t="s">
         <v>198</v>
@@ -12718,8 +12718,8 @@
       <c r="W21" t="s">
         <v>198</v>
       </c>
-      <c r="X21" t="s">
-        <v>198</v>
+      <c r="X21">
+        <v>0.52</v>
       </c>
       <c r="Y21" t="s">
         <v>198</v>
@@ -12916,8 +12916,8 @@
       <c r="CK21" t="s">
         <v>198</v>
       </c>
-      <c r="CL21" t="s">
-        <v>198</v>
+      <c r="CL21">
+        <v>21.11</v>
       </c>
       <c r="CM21" t="s">
         <v>198</v>
@@ -13281,14 +13281,14 @@
       <c r="R22" t="s">
         <v>198</v>
       </c>
-      <c r="S22" t="s">
-        <v>198</v>
+      <c r="S22">
+        <v>93.83</v>
       </c>
       <c r="T22" t="s">
         <v>198</v>
       </c>
-      <c r="U22" t="s">
-        <v>198</v>
+      <c r="U22">
+        <v>66.8</v>
       </c>
       <c r="V22" t="s">
         <v>198</v>
@@ -13296,8 +13296,8 @@
       <c r="W22" t="s">
         <v>198</v>
       </c>
-      <c r="X22" t="s">
-        <v>198</v>
+      <c r="X22">
+        <v>0.24</v>
       </c>
       <c r="Y22" t="s">
         <v>198</v>
@@ -13494,8 +13494,8 @@
       <c r="CK22" t="s">
         <v>198</v>
       </c>
-      <c r="CL22" t="s">
-        <v>198</v>
+      <c r="CL22">
+        <v>42.56</v>
       </c>
       <c r="CM22" t="s">
         <v>198</v>
@@ -13859,14 +13859,14 @@
       <c r="R23" t="s">
         <v>198</v>
       </c>
-      <c r="S23" t="s">
-        <v>198</v>
+      <c r="S23">
+        <v>34.02</v>
       </c>
       <c r="T23" t="s">
         <v>198</v>
       </c>
-      <c r="U23" t="s">
-        <v>198</v>
+      <c r="U23">
+        <v>31.43</v>
       </c>
       <c r="V23" t="s">
         <v>198</v>
@@ -13874,8 +13874,8 @@
       <c r="W23" t="s">
         <v>198</v>
       </c>
-      <c r="X23" t="s">
-        <v>198</v>
+      <c r="X23">
+        <v>0.92</v>
       </c>
       <c r="Y23" t="s">
         <v>198</v>
@@ -14072,8 +14072,8 @@
       <c r="CK23" t="s">
         <v>198</v>
       </c>
-      <c r="CL23" t="s">
-        <v>198</v>
+      <c r="CL23">
+        <v>35.5</v>
       </c>
       <c r="CM23" t="s">
         <v>198</v>
@@ -14437,14 +14437,14 @@
       <c r="R24" t="s">
         <v>198</v>
       </c>
-      <c r="S24" t="s">
-        <v>198</v>
+      <c r="S24">
+        <v>119.89</v>
       </c>
       <c r="T24" t="s">
         <v>198</v>
       </c>
-      <c r="U24" t="s">
-        <v>198</v>
+      <c r="U24">
+        <v>31.07</v>
       </c>
       <c r="V24" t="s">
         <v>198</v>
@@ -14452,8 +14452,8 @@
       <c r="W24" t="s">
         <v>198</v>
       </c>
-      <c r="X24" t="s">
-        <v>198</v>
+      <c r="X24">
+        <v>0.32</v>
       </c>
       <c r="Y24" t="s">
         <v>198</v>
@@ -14650,8 +14650,8 @@
       <c r="CK24" t="s">
         <v>198</v>
       </c>
-      <c r="CL24" t="s">
-        <v>198</v>
+      <c r="CL24">
+        <v>39.95</v>
       </c>
       <c r="CM24" t="s">
         <v>198</v>
@@ -15015,14 +15015,14 @@
       <c r="R25" t="s">
         <v>198</v>
       </c>
-      <c r="S25" t="s">
-        <v>198</v>
+      <c r="S25">
+        <v>146.78</v>
       </c>
       <c r="T25" t="s">
         <v>198</v>
       </c>
-      <c r="U25" t="s">
-        <v>198</v>
+      <c r="U25">
+        <v>50.43</v>
       </c>
       <c r="V25" t="s">
         <v>198</v>
@@ -15030,8 +15030,8 @@
       <c r="W25" t="s">
         <v>198</v>
       </c>
-      <c r="X25" t="s">
-        <v>198</v>
+      <c r="X25">
+        <v>0.05</v>
       </c>
       <c r="Y25" t="s">
         <v>198</v>
@@ -15228,8 +15228,8 @@
       <c r="CK25" t="s">
         <v>198</v>
       </c>
-      <c r="CL25" t="s">
-        <v>198</v>
+      <c r="CL25">
+        <v>44.53</v>
       </c>
       <c r="CM25" t="s">
         <v>198</v>
@@ -15593,14 +15593,14 @@
       <c r="R26" t="s">
         <v>198</v>
       </c>
-      <c r="S26" t="s">
-        <v>198</v>
+      <c r="S26">
+        <v>44.54</v>
       </c>
       <c r="T26" t="s">
         <v>198</v>
       </c>
-      <c r="U26" t="s">
-        <v>198</v>
+      <c r="U26">
+        <v>37.08</v>
       </c>
       <c r="V26" t="s">
         <v>198</v>
@@ -15608,8 +15608,8 @@
       <c r="W26" t="s">
         <v>198</v>
       </c>
-      <c r="X26" t="s">
-        <v>198</v>
+      <c r="X26">
+        <v>0.1</v>
       </c>
       <c r="Y26" t="s">
         <v>198</v>
@@ -15806,8 +15806,8 @@
       <c r="CK26" t="s">
         <v>198</v>
       </c>
-      <c r="CL26" t="s">
-        <v>198</v>
+      <c r="CL26">
+        <v>30.5</v>
       </c>
       <c r="CM26" t="s">
         <v>198</v>
@@ -16171,14 +16171,14 @@
       <c r="R27" t="s">
         <v>198</v>
       </c>
-      <c r="S27" t="s">
-        <v>198</v>
+      <c r="S27">
+        <v>148.17</v>
       </c>
       <c r="T27" t="s">
         <v>198</v>
       </c>
-      <c r="U27" t="s">
-        <v>198</v>
+      <c r="U27">
+        <v>32.59</v>
       </c>
       <c r="V27" t="s">
         <v>198</v>
@@ -16186,8 +16186,8 @@
       <c r="W27" t="s">
         <v>198</v>
       </c>
-      <c r="X27" t="s">
-        <v>198</v>
+      <c r="X27">
+        <v>0.45</v>
       </c>
       <c r="Y27" t="s">
         <v>198</v>
@@ -16384,8 +16384,8 @@
       <c r="CK27" t="s">
         <v>198</v>
       </c>
-      <c r="CL27" t="s">
-        <v>198</v>
+      <c r="CL27">
+        <v>19.53</v>
       </c>
       <c r="CM27" t="s">
         <v>198</v>
@@ -16749,14 +16749,14 @@
       <c r="R28" t="s">
         <v>198</v>
       </c>
-      <c r="S28" t="s">
-        <v>198</v>
+      <c r="S28">
+        <v>131.61</v>
       </c>
       <c r="T28" t="s">
         <v>198</v>
       </c>
-      <c r="U28" t="s">
-        <v>198</v>
+      <c r="U28">
+        <v>27.43</v>
       </c>
       <c r="V28" t="s">
         <v>198</v>
@@ -16764,8 +16764,8 @@
       <c r="W28" t="s">
         <v>198</v>
       </c>
-      <c r="X28" t="s">
-        <v>198</v>
+      <c r="X28">
+        <v>0.39</v>
       </c>
       <c r="Y28" t="s">
         <v>198</v>
@@ -16962,8 +16962,8 @@
       <c r="CK28" t="s">
         <v>198</v>
       </c>
-      <c r="CL28" t="s">
-        <v>198</v>
+      <c r="CL28">
+        <v>24.71</v>
       </c>
       <c r="CM28" t="s">
         <v>198</v>
@@ -17327,14 +17327,14 @@
       <c r="R29" t="s">
         <v>198</v>
       </c>
-      <c r="S29" t="s">
-        <v>198</v>
+      <c r="S29">
+        <v>131.25</v>
       </c>
       <c r="T29" t="s">
         <v>198</v>
       </c>
-      <c r="U29" t="s">
-        <v>198</v>
+      <c r="U29">
+        <v>43.95</v>
       </c>
       <c r="V29" t="s">
         <v>198</v>
@@ -17342,8 +17342,8 @@
       <c r="W29" t="s">
         <v>198</v>
       </c>
-      <c r="X29" t="s">
-        <v>198</v>
+      <c r="X29">
+        <v>0.63</v>
       </c>
       <c r="Y29" t="s">
         <v>198</v>
@@ -17540,8 +17540,8 @@
       <c r="CK29" t="s">
         <v>198</v>
       </c>
-      <c r="CL29" t="s">
-        <v>198</v>
+      <c r="CL29">
+        <v>35.9</v>
       </c>
       <c r="CM29" t="s">
         <v>198</v>
@@ -17905,14 +17905,14 @@
       <c r="R30" t="s">
         <v>198</v>
       </c>
-      <c r="S30" t="s">
-        <v>198</v>
+      <c r="S30">
+        <v>60.47</v>
       </c>
       <c r="T30" t="s">
         <v>198</v>
       </c>
-      <c r="U30" t="s">
-        <v>198</v>
+      <c r="U30">
+        <v>66.05</v>
       </c>
       <c r="V30" t="s">
         <v>198</v>
@@ -17920,8 +17920,8 @@
       <c r="W30" t="s">
         <v>198</v>
       </c>
-      <c r="X30" t="s">
-        <v>198</v>
+      <c r="X30">
+        <v>0.64</v>
       </c>
       <c r="Y30" t="s">
         <v>198</v>
@@ -18118,8 +18118,8 @@
       <c r="CK30" t="s">
         <v>198</v>
       </c>
-      <c r="CL30" t="s">
-        <v>198</v>
+      <c r="CL30">
+        <v>34.76</v>
       </c>
       <c r="CM30" t="s">
         <v>198</v>
@@ -18483,14 +18483,14 @@
       <c r="R31" t="s">
         <v>198</v>
       </c>
-      <c r="S31" t="s">
-        <v>198</v>
+      <c r="S31">
+        <v>127.7</v>
       </c>
       <c r="T31" t="s">
         <v>198</v>
       </c>
-      <c r="U31" t="s">
-        <v>198</v>
+      <c r="U31">
+        <v>37.03</v>
       </c>
       <c r="V31" t="s">
         <v>198</v>
@@ -18498,8 +18498,8 @@
       <c r="W31" t="s">
         <v>198</v>
       </c>
-      <c r="X31" t="s">
-        <v>198</v>
+      <c r="X31">
+        <v>0.72</v>
       </c>
       <c r="Y31" t="s">
         <v>198</v>
@@ -18696,8 +18696,8 @@
       <c r="CK31" t="s">
         <v>198</v>
       </c>
-      <c r="CL31" t="s">
-        <v>198</v>
+      <c r="CL31">
+        <v>23.81</v>
       </c>
       <c r="CM31" t="s">
         <v>198</v>
@@ -19061,14 +19061,14 @@
       <c r="R32" t="s">
         <v>198</v>
       </c>
-      <c r="S32" t="s">
-        <v>198</v>
+      <c r="S32">
+        <v>72.58</v>
       </c>
       <c r="T32" t="s">
         <v>198</v>
       </c>
-      <c r="U32" t="s">
-        <v>198</v>
+      <c r="U32">
+        <v>48.67</v>
       </c>
       <c r="V32" t="s">
         <v>198</v>
@@ -19076,8 +19076,8 @@
       <c r="W32" t="s">
         <v>198</v>
       </c>
-      <c r="X32" t="s">
-        <v>198</v>
+      <c r="X32">
+        <v>0.68</v>
       </c>
       <c r="Y32" t="s">
         <v>198</v>
@@ -19274,8 +19274,8 @@
       <c r="CK32" t="s">
         <v>198</v>
       </c>
-      <c r="CL32" t="s">
-        <v>198</v>
+      <c r="CL32">
+        <v>38.06</v>
       </c>
       <c r="CM32" t="s">
         <v>198</v>

</xml_diff>